<commit_message>
Change variables to undetermined
Available but need to request.
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-MSN.xlsx
+++ b/baseline/data_processing_elements-MSN.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\MSN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D814D6F9-E04B-4791-A9D9-2A5BBB89AA31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A537D76-AEEB-43BD-A9C1-F17B018B0AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="1840" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1726" uniqueCount="746">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1729" uniqueCount="747">
   <si>
     <t>index</t>
   </si>
@@ -1708,9 +1708,6 @@
     <t>Acceptable wording is "atrial fibrillation".</t>
   </si>
   <si>
-    <t>Minnesota_Afib_comb</t>
-  </si>
-  <si>
     <t>Minnesota classification of atrial fibrillation (persistent and intermittent combined)</t>
   </si>
   <si>
@@ -1777,12 +1774,6 @@
 If the study-specific variable was collected as part of a select-all-that-apply section without a response option for No, the harmonized values can be Yes/Presumed no. Code as "Presumed no" if the item was not selected but at least one other item in the section was selected.</t>
   </si>
   <si>
-    <t>B5_MS22.3b.2;
-B5_MS22.3b.4;
-B5_MS22.3b.5;
-B5_MS22.3b.7</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ever diagnosed: osteoarthritis;
 Ever diagnosed: rheumatoid arthritis;
 Ever diagnosed: psoriatic arthritis;
@@ -1798,10 +1789,6 @@
   </si>
   <si>
     <t>The "No" could not be generated because no "Other" category or variable.</t>
-  </si>
-  <si>
-    <t>case_when(B5_MS22.3b.2 == 1 | B5_MS22.3b.4 == 1 | B5_MS22.3b.5 == 1 | B5_MS22.3b.7 == 1 ~ 1L;
-ELSE ~ NA)</t>
   </si>
   <si>
     <t>dis_diabetes_ever</t>
@@ -2584,6 +2571,20 @@
   </si>
   <si>
     <t>participant ID</t>
+  </si>
+  <si>
+    <t>Available, would need to request.</t>
+  </si>
+  <si>
+    <t>Input variable Minnesota_Afib_comb. Would be direct_mapping.</t>
+  </si>
+  <si>
+    <t>Available but need to request.</t>
+  </si>
+  <si>
+    <t>Input variables B5_MS22.3b.2; B5_MS22.3b.4; B5_MS22.3b.5; B5_MS22.3b.7 available. 
+case_when(B5_MS22.3b.2 == 1 | B5_MS22.3b.4 == 1 | B5_MS22.3b.5 == 1 | B5_MS22.3b.7 == 1 ~ 1L;
+ELSE ~ NA)</t>
   </si>
 </sst>
 </file>
@@ -3049,45 +3050,45 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AG122"/>
-  <sheetFormatPr defaultColWidth="28.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="28.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" style="9" customWidth="1"/>
     <col min="2" max="2" width="7" style="9" customWidth="1"/>
-    <col min="3" max="3" width="28.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.81640625" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="39" style="9" customWidth="1"/>
-    <col min="5" max="5" width="45.42578125" style="9" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="45.453125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="12.453125" style="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.140625" style="9" customWidth="1"/>
-    <col min="10" max="10" width="28.7109375" style="9" customWidth="1"/>
-    <col min="11" max="11" width="18.42578125" style="9" customWidth="1"/>
+    <col min="8" max="8" width="15.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.1796875" style="9" customWidth="1"/>
+    <col min="10" max="10" width="28.7265625" style="9" customWidth="1"/>
+    <col min="11" max="11" width="18.453125" style="9" customWidth="1"/>
     <col min="12" max="12" width="37" style="10" customWidth="1"/>
-    <col min="13" max="13" width="33.5703125" style="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="32.7109375" style="9" customWidth="1"/>
-    <col min="15" max="15" width="16.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="56.140625" style="10" customWidth="1"/>
-    <col min="17" max="17" width="15.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="52.28515625" style="9" customWidth="1"/>
-    <col min="21" max="21" width="15.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="50.140625" style="10" customWidth="1"/>
-    <col min="23" max="23" width="21.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="27.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="28.28515625" style="9" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="33.54296875" style="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="32.7265625" style="9" customWidth="1"/>
+    <col min="15" max="15" width="16.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="56.1796875" style="10" customWidth="1"/>
+    <col min="17" max="17" width="15.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="52.26953125" style="9" customWidth="1"/>
+    <col min="21" max="21" width="15.453125" style="9" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="50.1796875" style="10" customWidth="1"/>
+    <col min="23" max="23" width="21.26953125" style="9" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="27.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="28.26953125" style="9" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="68" style="10" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="60.7109375" style="10" customWidth="1"/>
-    <col min="28" max="28" width="63.140625" style="10" customWidth="1"/>
-    <col min="29" max="29" width="60.7109375" style="10" customWidth="1"/>
+    <col min="27" max="27" width="60.7265625" style="10" customWidth="1"/>
+    <col min="28" max="28" width="63.1796875" style="10" customWidth="1"/>
+    <col min="29" max="29" width="60.7265625" style="10" customWidth="1"/>
     <col min="30" max="30" width="64" style="9" customWidth="1"/>
-    <col min="31" max="31" width="24.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="27.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="24.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="34" max="16384" width="28.7109375" style="9"/>
+    <col min="31" max="31" width="24.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="27.453125" style="9" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="24.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="34" max="16384" width="28.7265625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -3176,7 +3177,7 @@
         <v>28</v>
       </c>
       <c r="AD1" s="4" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="AE1" s="4" t="s">
         <v>29</v>
@@ -3188,7 +3189,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="9">
         <v>1</v>
       </c>
@@ -3216,10 +3217,10 @@
       <c r="K2" s="7"/>
       <c r="L2" s="8"/>
       <c r="M2" s="10" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="T2" s="10"/>
       <c r="W2" s="10" t="s">
@@ -3232,10 +3233,10 @@
         <v>40</v>
       </c>
       <c r="Z2" s="11" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="9">
         <v>2</v>
       </c>
@@ -3280,7 +3281,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="9">
         <v>3</v>
       </c>
@@ -3325,7 +3326,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="9">
         <v>4</v>
       </c>
@@ -3370,7 +3371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" s="9">
         <v>5</v>
       </c>
@@ -3424,7 +3425,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="7" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="9">
         <v>6</v>
       </c>
@@ -3473,7 +3474,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A8" s="9">
         <v>7</v>
       </c>
@@ -3524,7 +3525,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:33" ht="165" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A9" s="9">
         <v>8</v>
       </c>
@@ -3577,7 +3578,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="10" spans="1:33" ht="165" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A10" s="9">
         <v>9</v>
       </c>
@@ -3627,13 +3628,13 @@
         <v>76</v>
       </c>
       <c r="Z10" s="11" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="11" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="11" spans="1:33" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="9">
         <v>10</v>
       </c>
@@ -3688,7 +3689,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="12" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="9">
         <v>11</v>
       </c>
@@ -3727,7 +3728,7 @@
       <c r="N12" s="10"/>
       <c r="T12" s="10"/>
       <c r="V12" s="10" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
       <c r="W12" s="10" t="s">
         <v>117</v>
@@ -3742,7 +3743,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="9">
         <v>12</v>
       </c>
@@ -3781,7 +3782,7 @@
       <c r="N13" s="10"/>
       <c r="T13" s="10"/>
       <c r="V13" s="10" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="W13" s="10" t="s">
         <v>117</v>
@@ -3796,7 +3797,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="9">
         <v>13</v>
       </c>
@@ -3835,7 +3836,7 @@
       <c r="N14" s="10"/>
       <c r="T14" s="10"/>
       <c r="V14" s="10" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="W14" s="10" t="s">
         <v>117</v>
@@ -3850,7 +3851,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="15" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="9">
         <v>14</v>
       </c>
@@ -3889,7 +3890,7 @@
       <c r="N15" s="10"/>
       <c r="T15" s="10"/>
       <c r="V15" s="10" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="W15" s="10" t="s">
         <v>117</v>
@@ -3904,7 +3905,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="16" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="9">
         <v>15</v>
       </c>
@@ -3943,7 +3944,7 @@
       <c r="N16" s="10"/>
       <c r="T16" s="10"/>
       <c r="V16" s="10" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="W16" s="10" t="s">
         <v>117</v>
@@ -3958,7 +3959,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="17" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="9">
         <v>16</v>
       </c>
@@ -3997,7 +3998,7 @@
       <c r="N17" s="10"/>
       <c r="T17" s="10"/>
       <c r="V17" s="10" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="W17" s="10" t="s">
         <v>117</v>
@@ -4012,7 +4013,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="18" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="9">
         <v>17</v>
       </c>
@@ -4051,7 +4052,7 @@
       <c r="N18" s="10"/>
       <c r="T18" s="10"/>
       <c r="V18" s="10" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="W18" s="10" t="s">
         <v>117</v>
@@ -4066,7 +4067,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="19" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="9">
         <v>18</v>
       </c>
@@ -4105,7 +4106,7 @@
       <c r="N19" s="10"/>
       <c r="T19" s="10"/>
       <c r="V19" s="10" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="W19" s="10" t="s">
         <v>117</v>
@@ -4120,7 +4121,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="20" spans="1:30" ht="150" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" ht="145" x14ac:dyDescent="0.35">
       <c r="A20" s="9">
         <v>19</v>
       </c>
@@ -4174,16 +4175,16 @@
         <v>164</v>
       </c>
       <c r="AB20" s="14" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="AD20" s="9" t="s">
-        <v>729</v>
-      </c>
-    </row>
-    <row r="21" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="21" spans="1:30" ht="58" x14ac:dyDescent="0.35">
       <c r="A21" s="9">
         <v>20</v>
       </c>
@@ -4215,13 +4216,13 @@
         <v>170</v>
       </c>
       <c r="M21" s="14" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="N21" s="14" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
       <c r="P21" s="14" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="T21" s="10"/>
       <c r="W21" s="14" t="s">
@@ -4240,16 +4241,16 @@
         <v>172</v>
       </c>
       <c r="AB21" s="14" t="s">
-        <v>675</v>
+        <v>672</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="AD21" s="9" t="s">
-        <v>730</v>
-      </c>
-    </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="22" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A22" s="9">
         <v>21</v>
       </c>
@@ -4294,7 +4295,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="23" spans="1:30" ht="120" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" ht="116" x14ac:dyDescent="0.35">
       <c r="A23" s="9">
         <v>22</v>
       </c>
@@ -4320,19 +4321,19 @@
       <c r="K23" s="7"/>
       <c r="L23" s="8"/>
       <c r="M23" s="14" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>677</v>
+        <v>674</v>
       </c>
       <c r="P23" s="10" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="T23" s="10" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="V23" s="14" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
       <c r="W23" s="14" t="s">
         <v>171</v>
@@ -4350,16 +4351,16 @@
         <v>181</v>
       </c>
       <c r="AB23" s="14" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="AC23" s="10" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
       <c r="AD23" s="10" t="s">
-        <v>731</v>
-      </c>
-    </row>
-    <row r="24" spans="1:30" ht="150" x14ac:dyDescent="0.25">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="24" spans="1:30" ht="145" x14ac:dyDescent="0.35">
       <c r="A24" s="9">
         <v>23</v>
       </c>
@@ -4410,7 +4411,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="25" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A25" s="9">
         <v>24</v>
       </c>
@@ -4462,7 +4463,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="26" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A26" s="9">
         <v>25</v>
       </c>
@@ -4514,16 +4515,16 @@
         <v>202</v>
       </c>
       <c r="AB26" s="14" t="s">
-        <v>691</v>
+        <v>688</v>
       </c>
       <c r="AC26" s="10" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="AD26" s="9" t="s">
-        <v>732</v>
-      </c>
-    </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="27" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A27" s="9">
         <v>26</v>
       </c>
@@ -4574,7 +4575,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="28" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="9">
         <v>27</v>
       </c>
@@ -4619,7 +4620,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A29" s="9">
         <v>28</v>
       </c>
@@ -4670,7 +4671,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="9">
         <v>29</v>
       </c>
@@ -4715,7 +4716,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A31" s="9">
         <v>30</v>
       </c>
@@ -4766,7 +4767,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A32" s="9">
         <v>31</v>
       </c>
@@ -4820,7 +4821,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="33" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A33" s="9">
         <v>32</v>
       </c>
@@ -4865,7 +4866,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="34" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A34" s="9">
         <v>33</v>
       </c>
@@ -4912,7 +4913,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A35" s="9">
         <v>34</v>
       </c>
@@ -4957,7 +4958,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="36" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A36" s="9">
         <v>35</v>
       </c>
@@ -5013,7 +5014,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="37" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A37" s="9">
         <v>36</v>
       </c>
@@ -5067,7 +5068,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="38" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="9">
         <v>37</v>
       </c>
@@ -5121,7 +5122,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="39" spans="1:29" ht="90" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:29" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A39" s="9">
         <v>38</v>
       </c>
@@ -5175,7 +5176,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="40" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A40" s="9">
         <v>39</v>
       </c>
@@ -5220,7 +5221,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:29" ht="58" x14ac:dyDescent="0.35">
       <c r="A41" s="9">
         <v>40</v>
       </c>
@@ -5268,10 +5269,10 @@
         <v>290</v>
       </c>
       <c r="AC41" s="10" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="42" spans="1:29" x14ac:dyDescent="0.25">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="42" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A42" s="9">
         <v>41</v>
       </c>
@@ -5318,7 +5319,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="43" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A43" s="9">
         <v>42</v>
       </c>
@@ -5365,7 +5366,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="44" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A44" s="9">
         <v>43</v>
       </c>
@@ -5412,7 +5413,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="45" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A45" s="9">
         <v>44</v>
       </c>
@@ -5459,7 +5460,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="46" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:29" ht="58" x14ac:dyDescent="0.35">
       <c r="A46" s="9">
         <v>45</v>
       </c>
@@ -5511,7 +5512,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="47" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A47" s="9">
         <v>46</v>
       </c>
@@ -5558,7 +5559,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="48" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A48" s="9">
         <v>47</v>
       </c>
@@ -5610,7 +5611,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="49" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A49" s="9">
         <v>48</v>
       </c>
@@ -5663,7 +5664,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="50" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A50" s="9">
         <v>49</v>
       </c>
@@ -5713,10 +5714,10 @@
         <v>341</v>
       </c>
       <c r="AC50" s="10" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="51" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="51" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A51" s="9">
         <v>50</v>
       </c>
@@ -5772,7 +5773,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="52" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A52" s="9">
         <v>51</v>
       </c>
@@ -5821,7 +5822,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="53" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A53" s="9">
         <v>52</v>
       </c>
@@ -5873,7 +5874,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="54" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A54" s="9">
         <v>53</v>
       </c>
@@ -5923,16 +5924,16 @@
         <v>96</v>
       </c>
       <c r="Z54" s="12" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="AA54" s="10" t="s">
         <v>327</v>
       </c>
       <c r="AC54" s="10" t="s">
-        <v>728</v>
-      </c>
-    </row>
-    <row r="55" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="55" spans="1:30" ht="58" x14ac:dyDescent="0.35">
       <c r="A55" s="9">
         <v>54</v>
       </c>
@@ -5963,13 +5964,13 @@
         <v>370</v>
       </c>
       <c r="N55" s="10" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="T55" s="10" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
       <c r="V55" s="10" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="W55" s="10" t="s">
         <v>117</v>
@@ -5987,10 +5988,10 @@
         <v>371</v>
       </c>
       <c r="AC55" s="10" t="s">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="56" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="56" spans="1:30" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A56" s="9">
         <v>55</v>
       </c>
@@ -6043,13 +6044,13 @@
         <v>380</v>
       </c>
       <c r="AB56" s="14" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="AD56" s="9" t="s">
-        <v>733</v>
-      </c>
-    </row>
-    <row r="57" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="57" spans="1:30" ht="58" x14ac:dyDescent="0.35">
       <c r="A57" s="9">
         <v>56</v>
       </c>
@@ -6079,14 +6080,14 @@
         <v>383</v>
       </c>
       <c r="M57" s="10" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
       <c r="N57" s="10" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="T57" s="10"/>
       <c r="V57" s="10" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="W57" s="10" t="s">
         <v>117</v>
@@ -6104,10 +6105,10 @@
         <v>384</v>
       </c>
       <c r="AC57" s="10" t="s">
-        <v>717</v>
-      </c>
-    </row>
-    <row r="58" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="58" spans="1:30" ht="29" x14ac:dyDescent="0.35">
       <c r="A58" s="9">
         <v>57</v>
       </c>
@@ -6156,16 +6157,16 @@
         <v>171</v>
       </c>
       <c r="AB58" s="14" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="AC58" s="10" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="AD58" s="9" t="s">
-        <v>734</v>
-      </c>
-    </row>
-    <row r="59" spans="1:30" x14ac:dyDescent="0.25">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="59" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A59" s="9">
         <v>58</v>
       </c>
@@ -6210,7 +6211,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="1:30" ht="135" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:30" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A60" s="9">
         <v>59</v>
       </c>
@@ -6257,7 +6258,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="61" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:30" ht="29" x14ac:dyDescent="0.35">
       <c r="A61" s="9">
         <v>60</v>
       </c>
@@ -6304,7 +6305,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="62" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A62" s="9">
         <v>61</v>
       </c>
@@ -6351,7 +6352,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="63" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A63" s="9">
         <v>62</v>
       </c>
@@ -6396,7 +6397,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="64" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A64" s="9">
         <v>63</v>
       </c>
@@ -6441,7 +6442,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="65" spans="1:30" ht="165" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:30" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A65" s="9">
         <v>64</v>
       </c>
@@ -6486,7 +6487,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="66" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A66" s="9">
         <v>65</v>
       </c>
@@ -6533,7 +6534,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="67" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A67" s="9">
         <v>66</v>
       </c>
@@ -6580,7 +6581,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A68" s="9">
         <v>67</v>
       </c>
@@ -6627,7 +6628,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="69" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:30" ht="87" x14ac:dyDescent="0.35">
       <c r="A69" s="9">
         <v>68</v>
       </c>
@@ -6672,7 +6673,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="70" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:30" ht="58" x14ac:dyDescent="0.35">
       <c r="A70" s="9">
         <v>69</v>
       </c>
@@ -6705,10 +6706,10 @@
         <v>429</v>
       </c>
       <c r="N70" s="10" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="P70" s="10" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="S70" s="16"/>
       <c r="T70" s="14"/>
@@ -6728,16 +6729,16 @@
         <v>430</v>
       </c>
       <c r="AB70" s="14" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="AC70" s="10" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="AD70" s="10" t="s">
-        <v>735</v>
-      </c>
-    </row>
-    <row r="71" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="71" spans="1:30" ht="87" x14ac:dyDescent="0.35">
       <c r="A71" s="9">
         <v>70</v>
       </c>
@@ -6784,7 +6785,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="72" spans="1:30" ht="180" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:30" ht="174" x14ac:dyDescent="0.35">
       <c r="A72" s="9">
         <v>71</v>
       </c>
@@ -6816,16 +6817,16 @@
         <v>101</v>
       </c>
       <c r="M72" s="14" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="N72" s="10" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="P72" s="10" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="T72" s="10" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="V72" s="14"/>
       <c r="W72" s="14" t="s">
@@ -6844,16 +6845,16 @@
         <v>439</v>
       </c>
       <c r="AB72" s="14" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="AC72" s="10" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="AD72" s="10" t="s">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="73" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="73" spans="1:30" ht="29" x14ac:dyDescent="0.35">
       <c r="A73" s="9">
         <v>72</v>
       </c>
@@ -6900,7 +6901,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="74" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:30" ht="58" x14ac:dyDescent="0.35">
       <c r="A74" s="9">
         <v>73</v>
       </c>
@@ -6953,7 +6954,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="75" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:30" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A75" s="9">
         <v>74</v>
       </c>
@@ -6999,13 +7000,13 @@
         <v>458</v>
       </c>
       <c r="Z75" s="11" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="AC75" s="10" t="s">
-        <v>724</v>
-      </c>
-    </row>
-    <row r="76" spans="1:30" ht="409.5" x14ac:dyDescent="0.25">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="76" spans="1:30" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A76" s="9">
         <v>75</v>
       </c>
@@ -7049,13 +7050,13 @@
         <v>458</v>
       </c>
       <c r="Z76" s="11" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="AC76" s="10" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="77" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="77" spans="1:30" ht="87" x14ac:dyDescent="0.35">
       <c r="A77" s="9">
         <v>76</v>
       </c>
@@ -7106,7 +7107,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="78" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A78" s="9">
         <v>77</v>
       </c>
@@ -7141,10 +7142,10 @@
         <v>476</v>
       </c>
       <c r="N78" s="10" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="T78" s="10" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
       <c r="W78" s="10" t="s">
         <v>38</v>
@@ -7162,10 +7163,10 @@
         <v>478</v>
       </c>
       <c r="AD78" s="9" t="s">
-        <v>740</v>
-      </c>
-    </row>
-    <row r="79" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="79" spans="1:30" ht="58" x14ac:dyDescent="0.35">
       <c r="A79" s="9">
         <v>78</v>
       </c>
@@ -7217,13 +7218,13 @@
         <v>484</v>
       </c>
       <c r="AB79" s="14" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="AD79" s="10" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="80" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="80" spans="1:30" ht="58" x14ac:dyDescent="0.35">
       <c r="A80" s="9">
         <v>79</v>
       </c>
@@ -7279,13 +7280,13 @@
         <v>491</v>
       </c>
       <c r="AB80" s="14" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="AD80" s="10" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="81" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="81" spans="1:30" ht="58" x14ac:dyDescent="0.35">
       <c r="A81" s="9">
         <v>80</v>
       </c>
@@ -7341,13 +7342,13 @@
         <v>498</v>
       </c>
       <c r="AB81" s="14" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="AD81" s="10" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="82" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="82" spans="1:30" ht="58" x14ac:dyDescent="0.35">
       <c r="A82" s="9">
         <v>81</v>
       </c>
@@ -7403,13 +7404,13 @@
         <v>504</v>
       </c>
       <c r="AB82" s="14" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="AD82" s="10" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="83" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="83" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A83" s="9">
         <v>82</v>
       </c>
@@ -7458,7 +7459,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="84" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A84" s="9">
         <v>83</v>
       </c>
@@ -7490,28 +7491,34 @@
         <v>475</v>
       </c>
       <c r="M84" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="N84" s="10" t="s">
         <v>513</v>
       </c>
-      <c r="N84" s="10" t="s">
+      <c r="T84" s="10" t="s">
         <v>514</v>
       </c>
-      <c r="T84" s="10" t="s">
-        <v>515</v>
-      </c>
-      <c r="W84" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="X84" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y84" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="Z84" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="85" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+      <c r="W84" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="X84" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="Y84" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="Z84" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC84" s="10" t="s">
+        <v>744</v>
+      </c>
+      <c r="AD84" s="9" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="85" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A85" s="9">
         <v>84</v>
       </c>
@@ -7519,13 +7526,13 @@
         <v>32</v>
       </c>
       <c r="C85" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="D85" s="7" t="s">
         <v>516</v>
       </c>
-      <c r="D85" s="7" t="s">
+      <c r="E85" s="7" t="s">
         <v>517</v>
-      </c>
-      <c r="E85" s="7" t="s">
-        <v>518</v>
       </c>
       <c r="F85" s="7" t="s">
         <v>55</v>
@@ -7533,13 +7540,13 @@
       <c r="G85" s="7"/>
       <c r="H85" s="7"/>
       <c r="I85" s="7" t="s">
+        <v>518</v>
+      </c>
+      <c r="J85" s="7" t="s">
         <v>519</v>
       </c>
-      <c r="J85" s="7" t="s">
+      <c r="K85" s="7" t="s">
         <v>520</v>
-      </c>
-      <c r="K85" s="7" t="s">
-        <v>521</v>
       </c>
       <c r="L85" s="8" t="s">
         <v>475</v>
@@ -7562,13 +7569,13 @@
         <v>171</v>
       </c>
       <c r="AB85" s="14" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="AD85" s="10" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="86" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="86" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A86" s="9">
         <v>85</v>
       </c>
@@ -7576,13 +7583,13 @@
         <v>32</v>
       </c>
       <c r="C86" s="7" t="s">
+        <v>521</v>
+      </c>
+      <c r="D86" s="7" t="s">
         <v>522</v>
       </c>
-      <c r="D86" s="7" t="s">
+      <c r="E86" s="7" t="s">
         <v>523</v>
-      </c>
-      <c r="E86" s="7" t="s">
-        <v>524</v>
       </c>
       <c r="F86" s="7" t="s">
         <v>55</v>
@@ -7590,10 +7597,10 @@
       <c r="G86" s="7"/>
       <c r="H86" s="7"/>
       <c r="I86" s="7" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="J86" s="7" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="K86" s="7"/>
       <c r="L86" s="8" t="s">
@@ -7603,34 +7610,34 @@
         <v>45</v>
       </c>
       <c r="N86" s="10" t="s">
+        <v>525</v>
+      </c>
+      <c r="T86" s="10" t="s">
         <v>526</v>
       </c>
-      <c r="T86" s="10" t="s">
+      <c r="W86" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="X86" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="Y86" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="Z86" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="AA86" s="10" t="s">
         <v>527</v>
       </c>
-      <c r="W86" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="X86" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="Y86" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="Z86" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="AA86" s="10" t="s">
-        <v>528</v>
-      </c>
       <c r="AB86" s="14" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="AD86" s="10" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="87" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="87" spans="1:30" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A87" s="9">
         <v>86</v>
       </c>
@@ -7638,13 +7645,13 @@
         <v>32</v>
       </c>
       <c r="C87" s="7" t="s">
+        <v>528</v>
+      </c>
+      <c r="D87" s="7" t="s">
         <v>529</v>
       </c>
-      <c r="D87" s="7" t="s">
+      <c r="E87" s="7" t="s">
         <v>530</v>
-      </c>
-      <c r="E87" s="7" t="s">
-        <v>531</v>
       </c>
       <c r="F87" s="7" t="s">
         <v>55</v>
@@ -7653,38 +7660,41 @@
       <c r="H87" s="7"/>
       <c r="I87" s="7"/>
       <c r="J87" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K87" s="7"/>
       <c r="L87" s="8" t="s">
         <v>475</v>
       </c>
-      <c r="M87" s="10" t="s">
+      <c r="N87" s="10" t="s">
+        <v>532</v>
+      </c>
+      <c r="T87" s="10" t="s">
         <v>533</v>
       </c>
-      <c r="N87" s="10" t="s">
+      <c r="V87" s="10" t="s">
         <v>534</v>
       </c>
-      <c r="T87" s="10" t="s">
-        <v>535</v>
-      </c>
-      <c r="V87" s="10" t="s">
-        <v>536</v>
-      </c>
-      <c r="W87" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="X87" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y87" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="Z87" s="11" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="88" spans="1:30" ht="105" x14ac:dyDescent="0.25">
+      <c r="W87" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="X87" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="Y87" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="Z87" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC87" s="10" t="s">
+        <v>746</v>
+      </c>
+      <c r="AD87" s="9" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="88" spans="1:30" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A88" s="9">
         <v>87</v>
       </c>
@@ -7692,13 +7702,13 @@
         <v>32</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="D88" s="7" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="E88" s="7" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="F88" s="7" t="s">
         <v>55</v>
@@ -7706,25 +7716,25 @@
       <c r="G88" s="7"/>
       <c r="H88" s="7"/>
       <c r="I88" s="7" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="J88" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="K88" s="7" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="L88" s="8" t="s">
         <v>475</v>
       </c>
       <c r="M88" s="10" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="N88" s="10" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="T88" s="10" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="W88" s="10" t="s">
         <v>38</v>
@@ -7736,10 +7746,10 @@
         <v>76</v>
       </c>
       <c r="Z88" s="11" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="89" spans="1:30" ht="105" x14ac:dyDescent="0.25">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="89" spans="1:30" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A89" s="9">
         <v>88</v>
       </c>
@@ -7747,13 +7757,13 @@
         <v>32</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="D89" s="7" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="E89" s="7" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="F89" s="7" t="s">
         <v>55</v>
@@ -7763,19 +7773,19 @@
       <c r="I89" s="7"/>
       <c r="J89" s="7"/>
       <c r="K89" s="7" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="L89" s="8" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="M89" s="10" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="N89" s="10" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="T89" s="10" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="W89" s="10" t="s">
         <v>38</v>
@@ -7787,10 +7797,10 @@
         <v>76</v>
       </c>
       <c r="Z89" s="11" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="90" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="90" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A90" s="9">
         <v>89</v>
       </c>
@@ -7798,13 +7808,13 @@
         <v>32</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="D90" s="7" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="E90" s="7" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="F90" s="7" t="s">
         <v>55</v>
@@ -7813,10 +7823,10 @@
       <c r="H90" s="7"/>
       <c r="I90" s="7"/>
       <c r="J90" s="7" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="K90" s="7" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="L90" s="8" t="s">
         <v>475</v>
@@ -7825,10 +7835,10 @@
         <v>45</v>
       </c>
       <c r="N90" s="10" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="T90" s="10" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="W90" s="14" t="s">
         <v>171</v>
@@ -7843,16 +7853,16 @@
         <v>171</v>
       </c>
       <c r="AA90" s="10" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="AB90" s="14" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="AD90" s="9" t="s">
-        <v>742</v>
-      </c>
-    </row>
-    <row r="91" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="91" spans="1:30" ht="58" x14ac:dyDescent="0.35">
       <c r="A91" s="9">
         <v>90</v>
       </c>
@@ -7860,13 +7870,13 @@
         <v>32</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="D91" s="7" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="E91" s="7" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="F91" s="7" t="s">
         <v>55</v>
@@ -7875,7 +7885,7 @@
       <c r="H91" s="7"/>
       <c r="I91" s="7"/>
       <c r="J91" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K91" s="7"/>
       <c r="L91" s="8" t="s">
@@ -7899,19 +7909,19 @@
         <v>171</v>
       </c>
       <c r="AA91" s="10" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="AB91" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AC91" s="10" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="AD91" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="92" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="92" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A92" s="9">
         <v>91</v>
       </c>
@@ -7919,13 +7929,13 @@
         <v>32</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="D92" s="7" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="E92" s="7" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="F92" s="7" t="s">
         <v>55</v>
@@ -7934,7 +7944,7 @@
       <c r="H92" s="7"/>
       <c r="I92" s="7"/>
       <c r="J92" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K92" s="7"/>
       <c r="L92" s="8" t="s">
@@ -7958,13 +7968,13 @@
         <v>171</v>
       </c>
       <c r="AB92" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD92" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="93" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="93" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A93" s="9">
         <v>92</v>
       </c>
@@ -7972,13 +7982,13 @@
         <v>32</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="D93" s="7" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="E93" s="7" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="F93" s="7" t="s">
         <v>55</v>
@@ -7987,7 +7997,7 @@
       <c r="H93" s="7"/>
       <c r="I93" s="7"/>
       <c r="J93" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K93" s="7"/>
       <c r="L93" s="8" t="s">
@@ -8011,13 +8021,13 @@
         <v>171</v>
       </c>
       <c r="AB93" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD93" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="94" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="94" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A94" s="9">
         <v>93</v>
       </c>
@@ -8025,13 +8035,13 @@
         <v>32</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="D94" s="7" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="E94" s="7" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="F94" s="7" t="s">
         <v>55</v>
@@ -8040,7 +8050,7 @@
       <c r="H94" s="7"/>
       <c r="I94" s="7"/>
       <c r="J94" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K94" s="7"/>
       <c r="L94" s="8" t="s">
@@ -8064,13 +8074,13 @@
         <v>171</v>
       </c>
       <c r="AB94" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD94" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="95" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="95" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A95" s="9">
         <v>94</v>
       </c>
@@ -8078,13 +8088,13 @@
         <v>32</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="D95" s="7" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="E95" s="7" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="F95" s="7" t="s">
         <v>55</v>
@@ -8093,7 +8103,7 @@
       <c r="H95" s="7"/>
       <c r="I95" s="7"/>
       <c r="J95" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K95" s="7"/>
       <c r="L95" s="8" t="s">
@@ -8117,13 +8127,13 @@
         <v>171</v>
       </c>
       <c r="AB95" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD95" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="96" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="96" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A96" s="9">
         <v>95</v>
       </c>
@@ -8131,13 +8141,13 @@
         <v>32</v>
       </c>
       <c r="C96" s="7" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="D96" s="7" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="E96" s="7" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="F96" s="7" t="s">
         <v>55</v>
@@ -8146,7 +8156,7 @@
       <c r="H96" s="7"/>
       <c r="I96" s="7"/>
       <c r="J96" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K96" s="7"/>
       <c r="L96" s="8" t="s">
@@ -8170,13 +8180,13 @@
         <v>171</v>
       </c>
       <c r="AB96" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD96" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="97" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="97" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A97" s="9">
         <v>96</v>
       </c>
@@ -8184,13 +8194,13 @@
         <v>32</v>
       </c>
       <c r="C97" s="7" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="D97" s="7" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="E97" s="7" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="F97" s="7" t="s">
         <v>55</v>
@@ -8199,7 +8209,7 @@
       <c r="H97" s="7"/>
       <c r="I97" s="7"/>
       <c r="J97" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K97" s="7"/>
       <c r="L97" s="8" t="s">
@@ -8223,13 +8233,13 @@
         <v>171</v>
       </c>
       <c r="AB97" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD97" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="98" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="98" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A98" s="9">
         <v>97</v>
       </c>
@@ -8237,13 +8247,13 @@
         <v>32</v>
       </c>
       <c r="C98" s="7" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="D98" s="7" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="E98" s="7" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="F98" s="7" t="s">
         <v>55</v>
@@ -8252,7 +8262,7 @@
       <c r="H98" s="7"/>
       <c r="I98" s="7"/>
       <c r="J98" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K98" s="7"/>
       <c r="L98" s="8" t="s">
@@ -8276,13 +8286,13 @@
         <v>171</v>
       </c>
       <c r="AB98" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD98" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="99" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="99" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A99" s="9">
         <v>98</v>
       </c>
@@ -8290,13 +8300,13 @@
         <v>32</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="D99" s="7" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="E99" s="7" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="F99" s="7" t="s">
         <v>55</v>
@@ -8305,7 +8315,7 @@
       <c r="H99" s="7"/>
       <c r="I99" s="7"/>
       <c r="J99" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K99" s="7"/>
       <c r="L99" s="8" t="s">
@@ -8329,13 +8339,13 @@
         <v>171</v>
       </c>
       <c r="AB99" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD99" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="100" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="100" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A100" s="9">
         <v>99</v>
       </c>
@@ -8343,13 +8353,13 @@
         <v>32</v>
       </c>
       <c r="C100" s="7" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="D100" s="7" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="E100" s="7" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="F100" s="7" t="s">
         <v>55</v>
@@ -8358,7 +8368,7 @@
       <c r="H100" s="7"/>
       <c r="I100" s="7"/>
       <c r="J100" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K100" s="7"/>
       <c r="L100" s="8" t="s">
@@ -8382,13 +8392,13 @@
         <v>171</v>
       </c>
       <c r="AB100" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD100" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="101" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="101" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A101" s="9">
         <v>100</v>
       </c>
@@ -8396,13 +8406,13 @@
         <v>32</v>
       </c>
       <c r="C101" s="7" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="D101" s="7" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="E101" s="7" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="F101" s="7" t="s">
         <v>55</v>
@@ -8411,7 +8421,7 @@
       <c r="H101" s="7"/>
       <c r="I101" s="7"/>
       <c r="J101" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K101" s="7"/>
       <c r="L101" s="8" t="s">
@@ -8421,10 +8431,10 @@
         <v>45</v>
       </c>
       <c r="N101" s="10" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="T101" s="10" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="W101" s="14" t="s">
         <v>171</v>
@@ -8439,16 +8449,16 @@
         <v>171</v>
       </c>
       <c r="AA101" s="10" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="AB101" s="14" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="AD101" s="9" t="s">
-        <v>742</v>
-      </c>
-    </row>
-    <row r="102" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="102" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A102" s="9">
         <v>101</v>
       </c>
@@ -8456,13 +8466,13 @@
         <v>32</v>
       </c>
       <c r="C102" s="7" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="D102" s="7" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="E102" s="7" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="F102" s="7" t="s">
         <v>55</v>
@@ -8471,7 +8481,7 @@
       <c r="H102" s="7"/>
       <c r="I102" s="7"/>
       <c r="J102" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K102" s="7"/>
       <c r="L102" s="8" t="s">
@@ -8495,13 +8505,13 @@
         <v>171</v>
       </c>
       <c r="AB102" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD102" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="103" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="103" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A103" s="9">
         <v>102</v>
       </c>
@@ -8509,13 +8519,13 @@
         <v>32</v>
       </c>
       <c r="C103" s="7" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="D103" s="7" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="E103" s="7" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="F103" s="7" t="s">
         <v>55</v>
@@ -8524,7 +8534,7 @@
       <c r="H103" s="7"/>
       <c r="I103" s="7"/>
       <c r="J103" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K103" s="7"/>
       <c r="L103" s="8" t="s">
@@ -8548,13 +8558,13 @@
         <v>171</v>
       </c>
       <c r="AB103" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD103" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="104" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="104" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A104" s="9">
         <v>103</v>
       </c>
@@ -8562,13 +8572,13 @@
         <v>32</v>
       </c>
       <c r="C104" s="7" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="D104" s="7" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="E104" s="7" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="F104" s="7" t="s">
         <v>55</v>
@@ -8577,7 +8587,7 @@
       <c r="H104" s="7"/>
       <c r="I104" s="7"/>
       <c r="J104" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K104" s="7"/>
       <c r="L104" s="8" t="s">
@@ -8601,13 +8611,13 @@
         <v>171</v>
       </c>
       <c r="AB104" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD104" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="105" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="105" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A105" s="9">
         <v>104</v>
       </c>
@@ -8615,13 +8625,13 @@
         <v>32</v>
       </c>
       <c r="C105" s="7" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="D105" s="7" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="E105" s="7" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="F105" s="7" t="s">
         <v>55</v>
@@ -8630,7 +8640,7 @@
       <c r="H105" s="7"/>
       <c r="I105" s="7"/>
       <c r="J105" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K105" s="7"/>
       <c r="L105" s="8" t="s">
@@ -8654,13 +8664,13 @@
         <v>171</v>
       </c>
       <c r="AB105" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD105" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="106" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="106" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A106" s="9">
         <v>105</v>
       </c>
@@ -8668,13 +8678,13 @@
         <v>32</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="D106" s="7" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="E106" s="7" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="F106" s="7" t="s">
         <v>55</v>
@@ -8683,7 +8693,7 @@
       <c r="H106" s="7"/>
       <c r="I106" s="7"/>
       <c r="J106" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K106" s="7"/>
       <c r="L106" s="8" t="s">
@@ -8707,13 +8717,13 @@
         <v>171</v>
       </c>
       <c r="AB106" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD106" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="107" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="107" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A107" s="9">
         <v>106</v>
       </c>
@@ -8721,13 +8731,13 @@
         <v>32</v>
       </c>
       <c r="C107" s="7" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="D107" s="7" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="E107" s="7" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="F107" s="7" t="s">
         <v>55</v>
@@ -8736,7 +8746,7 @@
       <c r="H107" s="7"/>
       <c r="I107" s="7"/>
       <c r="J107" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K107" s="7"/>
       <c r="L107" s="8" t="s">
@@ -8760,13 +8770,13 @@
         <v>171</v>
       </c>
       <c r="AB107" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD107" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="108" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="108" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A108" s="9">
         <v>107</v>
       </c>
@@ -8774,13 +8784,13 @@
         <v>32</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D108" s="7" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="E108" s="7" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F108" s="7" t="s">
         <v>55</v>
@@ -8789,7 +8799,7 @@
       <c r="H108" s="7"/>
       <c r="I108" s="7"/>
       <c r="J108" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K108" s="7"/>
       <c r="L108" s="8" t="s">
@@ -8813,13 +8823,13 @@
         <v>171</v>
       </c>
       <c r="AB108" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD108" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="109" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="109" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A109" s="9">
         <v>108</v>
       </c>
@@ -8827,13 +8837,13 @@
         <v>32</v>
       </c>
       <c r="C109" s="7" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="D109" s="7" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="E109" s="7" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="F109" s="7" t="s">
         <v>55</v>
@@ -8842,7 +8852,7 @@
       <c r="H109" s="7"/>
       <c r="I109" s="7"/>
       <c r="J109" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="K109" s="7"/>
       <c r="L109" s="8" t="s">
@@ -8866,13 +8876,13 @@
         <v>171</v>
       </c>
       <c r="AB109" s="14" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AD109" s="10" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="110" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="110" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A110" s="9">
         <v>109</v>
       </c>
@@ -8880,13 +8890,13 @@
         <v>32</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="D110" s="7" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="E110" s="7" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="F110" s="7" t="s">
         <v>55</v>
@@ -8895,7 +8905,7 @@
       <c r="H110" s="7"/>
       <c r="I110" s="7"/>
       <c r="J110" s="7" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="K110" s="7"/>
       <c r="L110" s="8" t="s">
@@ -8919,7 +8929,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="111" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:30" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A111" s="9">
         <v>110</v>
       </c>
@@ -8927,13 +8937,13 @@
         <v>32</v>
       </c>
       <c r="C111" s="7" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="D111" s="7" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="E111" s="7" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="F111" s="7" t="s">
         <v>55</v>
@@ -8942,7 +8952,7 @@
       <c r="H111" s="7"/>
       <c r="I111" s="7"/>
       <c r="J111" s="7" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="K111" s="7"/>
       <c r="L111" s="8" t="s">
@@ -8952,10 +8962,10 @@
         <v>45</v>
       </c>
       <c r="N111" s="10" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="P111" s="10" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="T111" s="10"/>
       <c r="W111" s="14" t="s">
@@ -8971,13 +8981,13 @@
         <v>117</v>
       </c>
       <c r="AA111" s="10" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="AC111" s="14" t="s">
-        <v>713</v>
-      </c>
-    </row>
-    <row r="112" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="112" spans="1:30" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A112" s="9">
         <v>111</v>
       </c>
@@ -8985,13 +8995,13 @@
         <v>32</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="D112" s="7" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="E112" s="7" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="F112" s="7" t="s">
         <v>55</v>
@@ -9000,7 +9010,7 @@
       <c r="H112" s="7"/>
       <c r="I112" s="7"/>
       <c r="J112" s="7" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="K112" s="7"/>
       <c r="L112" s="8" t="s">
@@ -9024,7 +9034,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="113" spans="1:27" ht="45" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:27" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A113" s="9">
         <v>112</v>
       </c>
@@ -9032,13 +9042,13 @@
         <v>32</v>
       </c>
       <c r="C113" s="7" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="D113" s="7" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="E113" s="7" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="F113" s="7" t="s">
         <v>55</v>
@@ -9047,20 +9057,20 @@
       <c r="H113" s="7"/>
       <c r="I113" s="7"/>
       <c r="J113" s="7" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="K113" s="7"/>
       <c r="L113" s="8" t="s">
         <v>475</v>
       </c>
       <c r="M113" s="10" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="N113" s="10" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="T113" s="10" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="W113" s="10" t="s">
         <v>38</v>
@@ -9075,7 +9085,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="114" spans="1:27" ht="45" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:27" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A114" s="9">
         <v>113</v>
       </c>
@@ -9083,13 +9093,13 @@
         <v>32</v>
       </c>
       <c r="C114" s="7" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="D114" s="7" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="E114" s="7" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="F114" s="7" t="s">
         <v>55</v>
@@ -9098,20 +9108,20 @@
       <c r="H114" s="7"/>
       <c r="I114" s="7"/>
       <c r="J114" s="7" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="K114" s="7"/>
       <c r="L114" s="8" t="s">
         <v>475</v>
       </c>
       <c r="M114" s="10" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="N114" s="10" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="T114" s="10" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="W114" s="10" t="s">
         <v>38</v>
@@ -9126,7 +9136,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="115" spans="1:27" ht="45" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:27" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A115" s="9">
         <v>114</v>
       </c>
@@ -9134,13 +9144,13 @@
         <v>32</v>
       </c>
       <c r="C115" s="7" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="D115" s="7" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="E115" s="7" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="F115" s="7" t="s">
         <v>55</v>
@@ -9149,20 +9159,20 @@
       <c r="H115" s="7"/>
       <c r="I115" s="7"/>
       <c r="J115" s="7" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="K115" s="7"/>
       <c r="L115" s="8" t="s">
         <v>475</v>
       </c>
       <c r="M115" s="10" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="N115" s="10" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="T115" s="10" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="W115" s="10" t="s">
         <v>38</v>
@@ -9177,7 +9187,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="116" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A116" s="9">
         <v>115</v>
       </c>
@@ -9185,13 +9195,13 @@
         <v>32</v>
       </c>
       <c r="C116" s="7" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="D116" s="7" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="E116" s="7" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="F116" s="7" t="s">
         <v>55</v>
@@ -9200,7 +9210,7 @@
       <c r="H116" s="7"/>
       <c r="I116" s="7"/>
       <c r="J116" s="7" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="K116" s="7"/>
       <c r="L116" s="8"/>
@@ -9222,7 +9232,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="117" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A117" s="9">
         <v>116</v>
       </c>
@@ -9230,13 +9240,13 @@
         <v>32</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="D117" s="7" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="E117" s="7" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="F117" s="7" t="s">
         <v>55</v>
@@ -9245,7 +9255,7 @@
       <c r="H117" s="7"/>
       <c r="I117" s="7"/>
       <c r="J117" s="7" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="K117" s="7"/>
       <c r="L117" s="8"/>
@@ -9267,7 +9277,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="118" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A118" s="9">
         <v>117</v>
       </c>
@@ -9275,13 +9285,13 @@
         <v>32</v>
       </c>
       <c r="C118" s="7" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="D118" s="7" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="E118" s="7" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="F118" s="7" t="s">
         <v>55</v>
@@ -9290,7 +9300,7 @@
       <c r="H118" s="7"/>
       <c r="I118" s="7"/>
       <c r="J118" s="7" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="K118" s="7"/>
       <c r="L118" s="8"/>
@@ -9312,7 +9322,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="119" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A119" s="9">
         <v>118</v>
       </c>
@@ -9320,13 +9330,13 @@
         <v>32</v>
       </c>
       <c r="C119" s="7" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="D119" s="7" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="E119" s="7" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="F119" s="7" t="s">
         <v>55</v>
@@ -9335,7 +9345,7 @@
       <c r="H119" s="7"/>
       <c r="I119" s="7"/>
       <c r="J119" s="7" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="K119" s="7"/>
       <c r="L119" s="8"/>
@@ -9357,7 +9367,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="120" spans="1:27" ht="375" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:27" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A120" s="9">
         <v>119</v>
       </c>
@@ -9365,13 +9375,13 @@
         <v>32</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="D120" s="7" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="E120" s="7" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="F120" s="7" t="s">
         <v>55</v>
@@ -9380,18 +9390,18 @@
       <c r="H120" s="7"/>
       <c r="I120" s="7"/>
       <c r="J120" s="7" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="K120" s="7"/>
       <c r="L120" s="8"/>
       <c r="M120" s="10" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="N120" s="10" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="T120" s="10" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="W120" s="10" t="s">
         <v>38</v>
@@ -9403,13 +9413,13 @@
         <v>458</v>
       </c>
       <c r="Z120" s="12" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="AA120" s="10" t="s">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="121" spans="1:27" x14ac:dyDescent="0.25">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="121" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A121" s="9">
         <v>120</v>
       </c>
@@ -9417,13 +9427,13 @@
         <v>32</v>
       </c>
       <c r="C121" s="7" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="D121" s="7" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="E121" s="7" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="F121" s="7" t="s">
         <v>55</v>
@@ -9432,7 +9442,7 @@
       <c r="H121" s="7"/>
       <c r="I121" s="7"/>
       <c r="J121" s="7" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="K121" s="7"/>
       <c r="L121" s="8"/>
@@ -9454,7 +9464,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="122" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A122" s="9">
         <v>121</v>
       </c>
@@ -9462,13 +9472,13 @@
         <v>32</v>
       </c>
       <c r="C122" s="7" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="D122" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="E122" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="F122" s="7" t="s">
         <v>55</v>
@@ -9477,7 +9487,7 @@
       <c r="H122" s="7"/>
       <c r="I122" s="7"/>
       <c r="J122" s="7" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="K122" s="7"/>
       <c r="L122" s="8"/>

</xml_diff>